<commit_message>
electricity tariffs added, cameo costs to be updated
</commit_message>
<xml_diff>
--- a/Data/solar_prevalence_csiro_24.xlsx
+++ b/Data/solar_prevalence_csiro_24.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud-my.sharepoint.com/personal/dominic_jones_grattaninstitute_edu_au/Documents/Energy/Analysis/analysis_cp_dj_2025/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{E1A220D0-995B-4DF7-9C35-080FD36AC134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{440BC8B3-3FD2-4D72-AFCC-1EB984B127E1}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="8_{E1A220D0-995B-4DF7-9C35-080FD36AC134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{324EBF56-7295-446E-B182-51F5FBAE0148}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{A0DDE90D-8409-47C8-90CE-1E5B9CFF4EA4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{A0DDE90D-8409-47C8-90CE-1E5B9CFF4EA4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
   <si>
     <t>state</t>
   </si>
@@ -97,6 +98,18 @@
   </si>
   <si>
     <t>table A-1</t>
+  </si>
+  <si>
+    <t>pct_of_pv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proportion of PV systems with a battery </t>
+  </si>
+  <si>
+    <t>Figure 5-8</t>
+  </si>
+  <si>
+    <t>Scraped with webplotdigitiser</t>
   </si>
 </sst>
 </file>
@@ -734,4 +747,133 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BF5A529-99FF-4191-A4C1-3701B108F510}">
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>2024.9399074252201</v>
+      </c>
+      <c r="B2">
+        <v>0.132391042327131</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2029.43071578329</v>
+      </c>
+      <c r="B3">
+        <v>0.18552187256282199</v>
+      </c>
+      <c r="I3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>2033.9596276751899</v>
+      </c>
+      <c r="B4">
+        <v>0.25258307927601198</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>2038.88883937162</v>
+      </c>
+      <c r="B5">
+        <v>0.272849054501625</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>2043.4443690431499</v>
+      </c>
+      <c r="B6">
+        <v>0.27930660076369102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>2048.2282768330101</v>
+      </c>
+      <c r="B7">
+        <v>0.28999118817797798</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>2050.0391366440099</v>
+      </c>
+      <c r="B8">
+        <v>0.29668553949620602</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>2036.1672017907199</v>
+      </c>
+      <c r="B9">
+        <v>0.26699273784323002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>2031.90531849165</v>
+      </c>
+      <c r="B10">
+        <v>0.22163818861350501</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>2045.87758657361</v>
+      </c>
+      <c r="B11">
+        <v>0.28019710121440999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>2052.1855749460601</v>
+      </c>
+      <c r="B12">
+        <v>0.303257943300483</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>2053.2646889021598</v>
+      </c>
+      <c r="B13">
+        <v>0.30590817473741699</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>